<commit_message>
test: Fix typo in attribution test
</commit_message>
<xml_diff>
--- a/tests/integration/test_data/test_attribution.xlsx
+++ b/tests/integration/test_data/test_attribution.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Vidy/code/dnum/amendements-intelligents/tests/integration/test_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A9899B4-DA7D-5446-A8A9-800BB4E9EC41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9806D8E-9BE2-5E4A-BE47-E5C03AAB599D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="25600" windowHeight="28300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -84,13 +84,7 @@
     <t>article 5</t>
   </si>
   <si>
-    <t>I. – À la fin du I de l’article 313-20 du code d'mpositions sur les biens et services, les mots : « et dans une limite annuelle égale à 7 500 € » sont supprimés.</t>
-  </si>
-  <si>
     <t>article 6</t>
-  </si>
-  <si>
-    <t>I. – À la fin du I de l’article 314-24 du code d'mpositions sur les biens et services, les mots : « et dans une limite annuelle égale à 7 500 € » sont supprimés.</t>
   </si>
   <si>
     <t>article 7</t>
@@ -245,12 +239,18 @@
   <si>
     <t>1 ordonnance, 1 article, 1 expert</t>
   </si>
+  <si>
+    <t>I. – À la fin du I de l’article 313-20 du code d'impositions sur les biens et services, les mots : « et dans une limite annuelle égale à 7 500 € » sont supprimés.</t>
+  </si>
+  <si>
+    <t>I. – À la fin du I de l’article 314-24 du code d'impositions sur les biens et services, les mots : « et dans une limite annuelle égale à 7 500 € » sont supprimés.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -272,6 +272,12 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -307,7 +313,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -328,6 +334,9 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -681,8 +690,8 @@
       <c r="C6" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="D6" s="6" t="s">
-        <v>19</v>
+      <c r="D6" s="10" t="s">
+        <v>71</v>
       </c>
       <c r="E6" s="5" t="s">
         <v>9</v>
@@ -702,10 +711,10 @@
         <v>2694</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>21</v>
+        <v>19</v>
+      </c>
+      <c r="D7" s="10" t="s">
+        <v>72</v>
       </c>
       <c r="E7" s="5" t="s">
         <v>9</v>
@@ -744,16 +753,16 @@
         <v>2839</v>
       </c>
       <c r="C8" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="E8" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="F8" s="7" t="s">
         <v>23</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="F8" s="7" t="s">
-        <v>25</v>
       </c>
       <c r="G8" s="7" t="s">
         <v>11</v>
@@ -786,16 +795,16 @@
         <v>2862</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="G9" s="7" t="s">
         <v>11</v>
@@ -828,16 +837,16 @@
         <v>2863</v>
       </c>
       <c r="C10" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="E10" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="D10" s="6" t="s">
+      <c r="F10" s="7" t="s">
         <v>29</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="F10" s="7" t="s">
-        <v>31</v>
       </c>
       <c r="G10" s="7" t="s">
         <v>11</v>
@@ -870,16 +879,16 @@
         <v>2959</v>
       </c>
       <c r="C11" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="E11" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="D11" s="6" t="s">
+      <c r="F11" s="7" t="s">
         <v>33</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="F11" s="7" t="s">
-        <v>35</v>
       </c>
       <c r="G11" s="7" t="s">
         <v>11</v>
@@ -912,16 +921,16 @@
         <v>2967</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="G12" s="7" t="s">
         <v>11</v>
@@ -954,16 +963,16 @@
         <v>2971</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="G13" s="7" t="s">
         <v>11</v>
@@ -996,16 +1005,16 @@
         <v>2983</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="G14" s="7" t="s">
         <v>11</v>
@@ -1038,16 +1047,16 @@
         <v>3286</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="G15" s="7" t="s">
         <v>11</v>
@@ -1078,16 +1087,16 @@
         <v>3297</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="G16" s="7" t="s">
         <v>11</v>
@@ -1120,16 +1129,16 @@
         <v>3299</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="G17" s="7" t="s">
         <v>11</v>
@@ -1162,16 +1171,16 @@
         <v>3321</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F18" s="7" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="G18" s="7" t="s">
         <v>11</v>
@@ -1204,16 +1213,16 @@
         <v>3323</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="G19" s="7" t="s">
         <v>11</v>
@@ -1227,16 +1236,16 @@
         <v>3324</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F20" s="7" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="G20" s="7" t="s">
         <v>11</v>
@@ -1250,16 +1259,16 @@
         <v>3328</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="G21" s="7" t="s">
         <v>11</v>
@@ -1273,16 +1282,16 @@
         <v>3330</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F22" s="7" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="G22" s="7" t="s">
         <v>11</v>
@@ -1296,16 +1305,16 @@
         <v>3331</v>
       </c>
       <c r="C23" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="D23" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="E23" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="D23" s="6" t="s">
+      <c r="F23" s="7" t="s">
         <v>59</v>
-      </c>
-      <c r="E23" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="F23" s="7" t="s">
-        <v>61</v>
       </c>
       <c r="G23" s="7" t="s">
         <v>11</v>
@@ -1319,16 +1328,16 @@
         <v>3334</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F24" s="7" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="G24" s="7" t="s">
         <v>11</v>
@@ -1342,19 +1351,19 @@
         <v>3335</v>
       </c>
       <c r="C25" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="D25" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="E25" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="F25" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="G25" s="7" t="s">
         <v>64</v>
-      </c>
-      <c r="D25" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="E25" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="F25" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="G25" s="7" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="26" spans="1:26" ht="32" x14ac:dyDescent="0.2">
@@ -1365,19 +1374,19 @@
         <v>3336</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="F26" s="7" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="G26" s="7" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="27" spans="1:26" ht="32" x14ac:dyDescent="0.2">
@@ -1388,19 +1397,19 @@
         <v>3337</v>
       </c>
       <c r="C27" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="D27" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="D27" s="6" t="s">
-        <v>69</v>
-      </c>
       <c r="E27" s="5" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="F27" s="7" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="G27" s="7" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="28" spans="1:26" ht="32" x14ac:dyDescent="0.2">
@@ -1411,19 +1420,19 @@
         <v>3338</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="F28" s="7" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="G28" s="7" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="29" spans="1:26" ht="48" x14ac:dyDescent="0.2">
@@ -1434,19 +1443,19 @@
         <v>3339</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="F29" s="7" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="G29" s="7" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="30" spans="1:26" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
test: Add integration test for ignored sentences in attribution
</commit_message>
<xml_diff>
--- a/tests/integration/test_data/test_attribution.xlsx
+++ b/tests/integration/test_data/test_attribution.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11027"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11110"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Vidy/code/dnum/amendements-intelligents/tests/integration/test_data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Vidy/code/dnum/graal/tests/integration/test_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EC271D7-E81C-894E-B8D5-A97175BB4B8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7A9881D-8DED-2E4A-B798-C398A51536A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="25600" windowHeight="28300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="68800" windowHeight="28300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Amendements" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
feature: Add new attribution handler and use it for integration testing
</commit_message>
<xml_diff>
--- a/tests/integration/test_data/test_attribution.xlsx
+++ b/tests/integration/test_data/test_attribution.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Vidy/code/dnum/graal/tests/integration/test_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B84AF343-D9CE-9043-B2BC-AD76280763FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB75358C-4B12-7646-BD07-34EFF15C23A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="34400" windowHeight="28300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="51200" windowHeight="28300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Amendements" sheetId="1" r:id="rId1"/>
@@ -1963,10 +1963,10 @@
         <v>10</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="G30" s="5" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="H30" s="4" t="s">
         <v>126</v>

</xml_diff>

<commit_message>
test: Add tests for attribution handler and matchers
</commit_message>
<xml_diff>
--- a/tests/integration/test_data/test_attribution.xlsx
+++ b/tests/integration/test_data/test_attribution.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Vidy/code/dnum/graal/tests/integration/test_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB75358C-4B12-7646-BD07-34EFF15C23A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FB5ED06-0FD4-5C49-AF32-604E5CA22B75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="51200" windowHeight="28300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="331" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="134">
   <si>
     <t>amdt_idx</t>
   </si>
@@ -250,22 +250,6 @@
   </si>
   <si>
     <t>1 ordonnance, 1 article, 1 expert</t>
-  </si>
-  <si>
-    <t>article add. Ap 3</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Le code de la sécurité sociale est ainsi modifié :
-  1° Le III de l’article L. 137-16 est complété par un 9° ainsi rédigé :
-  « 9° Les rémunérations et éléments de rémunération mentionnés à l’article L. 137-16 du présent code. » ;
-  2° L’article L. 241-13 est ainsi rédigé :
-  « Art. L. 241-13. – I. – Toute heure supplémentaire effectuée par les salariés mentionnés au I de l’article L. 137-16 ouvre droit à une déduction forfaitaire des cotisations patronales à hauteur d’un montant fixé par décret. Ce montant peut être majoré dans les entreprises employant au plus vingt salariés »
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">- 1 code : Le code de la sécurité sociale 
-- 2 experts : Marie Faugeron et Marin Guédo-Guilloteau
-- Pas de mot clé </t>
   </si>
   <si>
     <t>article add. Ap 4</t>
@@ -870,7 +854,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:AB991"/>
+  <dimension ref="A1:AB990"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.5" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="4" max="5" width="60.1640625" customWidth="1"/>
@@ -902,7 +886,7 @@
         <v>6</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="I1" s="2" t="s">
         <v>7</v>
@@ -931,7 +915,7 @@
         <v>12</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="I2" s="5" t="s">
         <v>13</v>
@@ -960,7 +944,7 @@
         <v>12</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="I3" s="5" t="s">
         <v>13</v>
@@ -989,7 +973,7 @@
         <v>12</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="I4" s="5" t="s">
         <v>13</v>
@@ -1018,7 +1002,7 @@
         <v>12</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="I5" s="5" t="s">
         <v>13</v>
@@ -1047,7 +1031,7 @@
         <v>12</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="I6" s="5" t="s">
         <v>13</v>
@@ -1076,7 +1060,7 @@
         <v>12</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="I7" s="5" t="s">
         <v>13</v>
@@ -1124,7 +1108,7 @@
         <v>27</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="I8" s="5" t="s">
         <v>13</v>
@@ -1172,7 +1156,7 @@
         <v>27</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="I9" s="5" t="s">
         <v>13</v>
@@ -1220,7 +1204,7 @@
         <v>33</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="I10" s="5" t="s">
         <v>13</v>
@@ -1268,7 +1252,7 @@
         <v>37</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="I11" s="5" t="s">
         <v>13</v>
@@ -1316,7 +1300,7 @@
         <v>37</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="I12" s="5" t="s">
         <v>13</v>
@@ -1364,7 +1348,7 @@
         <v>37</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="I13" s="5" t="s">
         <v>13</v>
@@ -1412,7 +1396,7 @@
         <v>37</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="I14" s="5" t="s">
         <v>13</v>
@@ -1460,7 +1444,7 @@
         <v>37</v>
       </c>
       <c r="H15" s="4" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="I15" s="5" t="s">
         <v>13</v>
@@ -1506,7 +1490,7 @@
         <v>37</v>
       </c>
       <c r="H16" s="4" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="I16" s="5" t="s">
         <v>13</v>
@@ -1554,7 +1538,7 @@
         <v>37</v>
       </c>
       <c r="H17" s="4" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="I17" s="5" t="s">
         <v>13</v>
@@ -1602,7 +1586,7 @@
         <v>37</v>
       </c>
       <c r="H18" s="4" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="I18" s="5" t="s">
         <v>13</v>
@@ -1650,7 +1634,7 @@
         <v>27</v>
       </c>
       <c r="H19" s="4" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="I19" s="5" t="s">
         <v>13</v>
@@ -1679,7 +1663,7 @@
         <v>37</v>
       </c>
       <c r="H20" s="4" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="I20" s="5" t="s">
         <v>13</v>
@@ -1708,7 +1692,7 @@
         <v>37</v>
       </c>
       <c r="H21" s="4" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="I21" s="5" t="s">
         <v>13</v>
@@ -1737,7 +1721,7 @@
         <v>37</v>
       </c>
       <c r="H22" s="4" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="I22" s="5" t="s">
         <v>13</v>
@@ -1766,7 +1750,7 @@
         <v>63</v>
       </c>
       <c r="H23" s="4" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="I23" s="5" t="s">
         <v>13</v>
@@ -1795,7 +1779,7 @@
         <v>37</v>
       </c>
       <c r="H24" s="4" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="I24" s="5" t="s">
         <v>13</v>
@@ -1824,7 +1808,7 @@
         <v>27</v>
       </c>
       <c r="H25" s="4" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="I25" s="5" t="s">
         <v>68</v>
@@ -1853,7 +1837,7 @@
         <v>63</v>
       </c>
       <c r="H26" s="4" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="I26" s="5" t="s">
         <v>68</v>
@@ -1882,7 +1866,7 @@
         <v>63</v>
       </c>
       <c r="H27" s="4" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="I27" s="5" t="s">
         <v>68</v>
@@ -1911,7 +1895,7 @@
         <v>27</v>
       </c>
       <c r="H28" s="4" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="I28" s="5" t="s">
         <v>68</v>
@@ -1940,7 +1924,7 @@
         <v>27</v>
       </c>
       <c r="H29" s="4" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="I29" s="5" t="s">
         <v>74</v>
@@ -1962,20 +1946,20 @@
       <c r="E30" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="F30" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="G30" s="5" t="s">
-        <v>33</v>
+      <c r="F30" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G30" s="8" t="s">
+        <v>12</v>
       </c>
       <c r="H30" s="4" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="I30" s="5" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="31" spans="1:28" ht="64" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:28" ht="48" x14ac:dyDescent="0.2">
       <c r="A31" s="3">
         <v>30</v>
       </c>
@@ -1991,20 +1975,20 @@
       <c r="E31" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="F31" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="G31" s="8" t="s">
-        <v>12</v>
+      <c r="F31" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G31" s="5" t="s">
+        <v>27</v>
       </c>
       <c r="H31" s="4" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="I31" s="5" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="32" spans="1:28" ht="48" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:28" ht="144" x14ac:dyDescent="0.2">
       <c r="A32" s="3">
         <v>31</v>
       </c>
@@ -2014,26 +1998,26 @@
       <c r="C32" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="D32" s="6" t="s">
+      <c r="D32" s="7" t="s">
         <v>82</v>
       </c>
       <c r="E32" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="F32" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="G32" s="5" t="s">
-        <v>27</v>
+      <c r="F32" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G32" s="8" t="s">
+        <v>12</v>
       </c>
       <c r="H32" s="4" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="I32" s="5" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="33" spans="1:9" ht="144" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:9" ht="112" x14ac:dyDescent="0.2">
       <c r="A33" s="3">
         <v>32</v>
       </c>
@@ -2043,17 +2027,17 @@
       <c r="C33" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="D33" s="7" t="s">
+      <c r="D33" s="4" t="s">
         <v>85</v>
       </c>
       <c r="E33" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="F33" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="G33" s="8" t="s">
-        <v>12</v>
+      <c r="F33" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="G33" s="5" t="s">
+        <v>90</v>
       </c>
       <c r="H33" s="4" t="s">
         <v>125</v>
@@ -2062,7 +2046,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="34" spans="1:9" ht="112" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:9" ht="144" x14ac:dyDescent="0.2">
       <c r="A34" s="3">
         <v>33</v>
       </c>
@@ -2072,26 +2056,26 @@
       <c r="C34" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="D34" s="4" t="s">
+      <c r="D34" s="7" t="s">
         <v>88</v>
       </c>
       <c r="E34" s="4" t="s">
         <v>10</v>
       </c>
       <c r="F34" s="4" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="G34" s="5" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="H34" s="4" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="I34" s="5" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="35" spans="1:9" ht="144" x14ac:dyDescent="0.2">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" ht="240" x14ac:dyDescent="0.2">
       <c r="A35" s="3">
         <v>34</v>
       </c>
@@ -2099,28 +2083,28 @@
         <v>34</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D35" s="7" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="E35" s="4" t="s">
         <v>10</v>
       </c>
       <c r="F35" s="4" t="s">
-        <v>92</v>
+        <v>26</v>
       </c>
       <c r="G35" s="5" t="s">
-        <v>93</v>
+        <v>27</v>
       </c>
       <c r="H35" s="4" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="I35" s="5" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="36" spans="1:9" ht="240" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:9" ht="144" x14ac:dyDescent="0.2">
       <c r="A36" s="3">
         <v>35</v>
       </c>
@@ -2136,14 +2120,14 @@
       <c r="E36" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="F36" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="G36" s="5" t="s">
-        <v>27</v>
+      <c r="F36" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G36" s="8" t="s">
+        <v>12</v>
       </c>
       <c r="H36" s="4" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="I36" s="5" t="s">
         <v>97</v>
@@ -2172,13 +2156,13 @@
         <v>12</v>
       </c>
       <c r="H37" s="4" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="I37" s="5" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="38" spans="1:9" ht="144" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:9" ht="208" x14ac:dyDescent="0.2">
       <c r="A38" s="3">
         <v>37</v>
       </c>
@@ -2201,7 +2185,7 @@
         <v>12</v>
       </c>
       <c r="H38" s="4" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="I38" s="5" t="s">
         <v>103</v>
@@ -2215,10 +2199,10 @@
         <v>38</v>
       </c>
       <c r="C39" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="D39" s="7" t="s">
         <v>104</v>
-      </c>
-      <c r="D39" s="7" t="s">
-        <v>105</v>
       </c>
       <c r="E39" s="4" t="s">
         <v>10</v>
@@ -2230,13 +2214,13 @@
         <v>12</v>
       </c>
       <c r="H39" s="4" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="I39" s="5" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="40" spans="1:9" ht="208" x14ac:dyDescent="0.2">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A40" s="3">
         <v>39</v>
       </c>
@@ -2244,86 +2228,86 @@
         <v>39</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="D40" s="7" t="s">
-        <v>107</v>
+        <v>101</v>
+      </c>
+      <c r="D40" s="4" t="s">
+        <v>105</v>
       </c>
       <c r="E40" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="F40" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="G40" s="8" t="s">
-        <v>12</v>
+      <c r="F40" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="G40" s="5" t="s">
+        <v>107</v>
       </c>
       <c r="H40" s="4" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="I40" s="5" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="41" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" ht="48" x14ac:dyDescent="0.2">
       <c r="A41" s="3">
         <v>40</v>
       </c>
-      <c r="B41" s="4">
+      <c r="B41" s="3">
         <v>40</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="D41" s="4" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E41" s="4" t="s">
         <v>10</v>
       </c>
       <c r="F41" s="9" t="s">
-        <v>109</v>
+        <v>89</v>
       </c>
       <c r="G41" s="5" t="s">
-        <v>110</v>
+        <v>90</v>
       </c>
       <c r="H41" s="4" t="s">
         <v>125</v>
       </c>
       <c r="I41" s="5" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="42" spans="1:9" ht="48" x14ac:dyDescent="0.2">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" ht="112" x14ac:dyDescent="0.2">
       <c r="A42" s="3">
         <v>41</v>
       </c>
-      <c r="B42" s="4">
+      <c r="B42" s="3">
         <v>41</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="D42" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="D42" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="E42" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="E42" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="F42" s="9" t="s">
-        <v>92</v>
+      <c r="F42" s="4" t="s">
+        <v>26</v>
       </c>
       <c r="G42" s="5" t="s">
-        <v>93</v>
+        <v>27</v>
       </c>
       <c r="H42" s="4" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="I42" s="5" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="43" spans="1:9" ht="112" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:9" ht="176" x14ac:dyDescent="0.2">
       <c r="A43" s="3">
         <v>42</v>
       </c>
@@ -2331,28 +2315,28 @@
         <v>42</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="D43" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="E43" s="4" t="s">
         <v>114</v>
       </c>
-      <c r="E43" s="4" t="s">
+      <c r="F43" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G43" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="H43" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="I43" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="F43" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="G43" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="H43" s="4" t="s">
-        <v>126</v>
-      </c>
-      <c r="I43" s="5" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="44" spans="1:9" ht="176" x14ac:dyDescent="0.2">
+    </row>
+    <row r="44" spans="1:9" ht="144" x14ac:dyDescent="0.2">
       <c r="A44" s="3">
         <v>43</v>
       </c>
@@ -2360,28 +2344,28 @@
         <v>43</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="D44" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="E44" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="F44" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="G44" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="H44" s="4" t="s">
         <v>124</v>
       </c>
-      <c r="E44" s="4" t="s">
-        <v>117</v>
-      </c>
-      <c r="F44" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="G44" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="H44" s="4" t="s">
-        <v>125</v>
-      </c>
       <c r="I44" s="5" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="45" spans="1:9" ht="144" x14ac:dyDescent="0.2">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A45" s="3">
         <v>44</v>
       </c>
@@ -2389,13 +2373,13 @@
         <v>44</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="D45" s="7" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="E45" s="4" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="F45" s="4" t="s">
         <v>36</v>
@@ -2404,69 +2388,49 @@
         <v>37</v>
       </c>
       <c r="H45" s="4" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="I45" s="5" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="46" spans="1:9" ht="32" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:9" ht="64" x14ac:dyDescent="0.2">
       <c r="A46" s="3">
         <v>45</v>
       </c>
       <c r="B46" s="3">
-        <v>44</v>
-      </c>
-      <c r="C46" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="D46" s="7" t="s">
-        <v>120</v>
-      </c>
-      <c r="E46" s="4" t="s">
-        <v>121</v>
-      </c>
-      <c r="F46" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="G46" s="5" t="s">
-        <v>37</v>
+        <v>45</v>
+      </c>
+      <c r="C46" t="s">
+        <v>127</v>
+      </c>
+      <c r="D46" t="s">
+        <v>128</v>
+      </c>
+      <c r="E46" t="s">
+        <v>129</v>
+      </c>
+      <c r="F46" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="G46" t="s">
+        <v>130</v>
       </c>
       <c r="H46" s="4" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="I46" s="5" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="47" spans="1:9" ht="64" x14ac:dyDescent="0.2">
-      <c r="A47" s="3">
-        <v>46</v>
-      </c>
-      <c r="B47" s="4">
-        <v>45</v>
-      </c>
-      <c r="C47" t="s">
-        <v>130</v>
-      </c>
-      <c r="D47" t="s">
-        <v>131</v>
-      </c>
-      <c r="E47" t="s">
-        <v>132</v>
-      </c>
-      <c r="F47" s="10" t="s">
-        <v>134</v>
-      </c>
-      <c r="G47" t="s">
         <v>133</v>
       </c>
-      <c r="H47" s="4" t="s">
-        <v>135</v>
-      </c>
-      <c r="I47" s="5" t="s">
-        <v>136</v>
-      </c>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="B47" s="4"/>
+      <c r="C47" s="4"/>
+      <c r="D47" s="4"/>
+      <c r="E47" s="4"/>
+      <c r="F47" s="4"/>
+      <c r="G47" s="5"/>
+      <c r="I47" s="5"/>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B48" s="4"/>
@@ -2474,7 +2438,6 @@
       <c r="D48" s="4"/>
       <c r="E48" s="4"/>
       <c r="F48" s="4"/>
-      <c r="G48" s="5"/>
       <c r="I48" s="5"/>
     </row>
     <row r="49" spans="2:9" x14ac:dyDescent="0.2">
@@ -2483,6 +2446,7 @@
       <c r="D49" s="4"/>
       <c r="E49" s="4"/>
       <c r="F49" s="4"/>
+      <c r="G49" s="5"/>
       <c r="I49" s="5"/>
     </row>
     <row r="50" spans="2:9" x14ac:dyDescent="0.2">
@@ -10954,20 +10918,11 @@
       <c r="G990" s="5"/>
       <c r="I990" s="5"/>
     </row>
-    <row r="991" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B991" s="4"/>
-      <c r="C991" s="4"/>
-      <c r="D991" s="4"/>
-      <c r="E991" s="4"/>
-      <c r="F991" s="4"/>
-      <c r="G991" s="5"/>
-      <c r="I991" s="5"/>
-    </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="F41" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-    <hyperlink ref="F42" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
-    <hyperlink ref="F47" r:id="rId3" xr:uid="{2ED7B83F-1573-4B4A-B81D-6D42EFEEE2A6}"/>
+    <hyperlink ref="F40" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="F41" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="F46" r:id="rId3" xr:uid="{2ED7B83F-1573-4B4A-B81D-6D42EFEEE2A6}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>

</xml_diff>

<commit_message>
fix: Attribution tests for attribution
</commit_message>
<xml_diff>
--- a/tests/integration/test_data/test_attribution.xlsx
+++ b/tests/integration/test_data/test_attribution.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10209"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10824"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Vidy/code/dnum/graal/tests/integration/test_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54287306-DE41-1646-AB1B-137E6175E1BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17178D82-FE9B-334A-8DC9-82E867F1D780}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25600" yWindow="500" windowWidth="25600" windowHeight="28300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="51200" windowHeight="28300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Amendements" sheetId="1" r:id="rId1"/>
@@ -63,9 +63,6 @@
     <t>julien.dauce@sante.gouv.fr</t>
   </si>
   <si>
-    <t>Julien Dauce</t>
-  </si>
-  <si>
     <t>1 code, 1 article, 1 expert</t>
   </si>
   <si>
@@ -108,9 +105,6 @@
     <t>marie.faugeron@sante.gouv.fr</t>
   </si>
   <si>
-    <t>Marie Faugeron</t>
-  </si>
-  <si>
     <t>article 8</t>
   </si>
   <si>
@@ -126,9 +120,6 @@
     <t>marin.guedo-guilloteau@sante.gouv.fr</t>
   </si>
   <si>
-    <t>Marin Guédo-Guilloteau</t>
-  </si>
-  <si>
     <t>article 10</t>
   </si>
   <si>
@@ -138,9 +129,6 @@
     <t>nathan.soto@sante.gouv.fr</t>
   </si>
   <si>
-    <t>Nathan Soto</t>
-  </si>
-  <si>
     <t>article 11</t>
   </si>
   <si>
@@ -214,9 +202,6 @@
   </si>
   <si>
     <t>margot.cavely@sante.gouv.fr</t>
-  </si>
-  <si>
-    <t>Margot Cavely</t>
   </si>
   <si>
     <t>article 23</t>
@@ -259,11 +244,6 @@
 II. – Le code du service national est ainsi modifié :
 Le III de l’article L. 0121-2-1 est complété par un 9° ainsi rédigé :
   « 9° Les rémunérations et éléments de rémunération mentionnés à l’article L. 0121-2-1 du présent code. » ;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">- 2 codes : Le code général des impôts, le code du service national 
-- 2 experts : Julien Dauce, Nathan Soto
-- Pas de mot clé </t>
   </si>
   <si>
     <t>article add. Ap 5</t>
@@ -322,9 +302,6 @@
     <t>etienne.barraud@sante.gouv.fr</t>
   </si>
   <si>
-    <t>Etienne Barraud</t>
-  </si>
-  <si>
     <t>- 2 codes : code général des impôts, code des Impositions sur les biens et services
 - Pas d'experts correspondants
 - Pas de mot clé 
@@ -342,12 +319,6 @@
 </t>
   </si>
   <si>
-    <t>- 1 code : Le code de la sécurité sociale 
-- 2 experts : Marie Faugeron et Marin Guédo-Guilloteau
-- 1 mot clé : cotisations de l'employeur
-- 1 expert : Marie Faugeron</t>
-  </si>
-  <si>
     <t>article add. Ap 10</t>
   </si>
   <si>
@@ -357,12 +328,6 @@
   « 9° Les composants de salaire mentionnés à l’article L. 0121-2-1 du présent code. » ;</t>
   </si>
   <si>
-    <t xml:space="preserve">- 2 codes : Le code général des impôts, le code du service national 
-- 2 experts : Julien Dauce, Nathan Soto
-- 1 mot-clé : composants de salaire
-- 1 expert </t>
-  </si>
-  <si>
     <t>article add. Ap 11</t>
   </si>
   <si>
@@ -370,12 +335,6 @@
 II. – Le code du service national est ainsi modifié :
 Le III de l’article L. 0121-2-1 est complété par un 9° ainsi rédigé :
   « 9° Les composants de salaire établis par un organisme de protection sociale mentionnés à l’article L. 0121-2-1 du présent code. » ;</t>
-  </si>
-  <si>
-    <t>- 2 codes : Le code général des impôts, le code du service national 
-- 2 experts : Julien Dauce, Nathan Soto
-- 2 mot-clés : composants de salaire, organisme de protection sociale
-- 2 experts : Julien Dauce, Nathan Soto</t>
   </si>
   <si>
     <t>article add. Ap 12</t>
@@ -388,13 +347,6 @@
 II. – La perte de recettes pour l’État est compensée à due concurrence par la création d’une taxe additionnelle à l’accise sur les tabacs prévue au chapitre IV du titre Ier du livre III du code des impositions sur les biens et services.</t>
   </si>
   <si>
-    <t xml:space="preserve">- 2 codes : Le code général des impôts, le code du service national 
-- 2 experts : Julien Dauce, Nathan Soto
-- 2 mot-clés : composants de salaire, tabac
-- 2 ème mot clé dans une phrase ignorée 
-- 1 expert </t>
-  </si>
-  <si>
     <t>I. – À la fin du I de l’article 1635 bis du code général des impôts, les mots : « et dans une limite annuelle égale à 7 500 € » sont supprimés.
 II. – Le code du service national est ainsi modifié :
 Le III de l’article L. 0121-2-1 est complété par un 9° ainsi rédigé :
@@ -408,16 +360,10 @@
     <t>jmm@sante.gouv.fr</t>
   </si>
   <si>
-    <t>Jean-Michel Montant</t>
-  </si>
-  <si>
     <t>- Montant M</t>
   </si>
   <si>
     <t>Ici on parle de montant A et de montant Merveilleux parce que ça commence par M</t>
-  </si>
-  <si>
-    <t>- Autres montants mais on ne souhaite pas les voir attribués à Jean-Michel Montant puisque ce ne sont pas des montants M ou Z</t>
   </si>
   <si>
     <t xml:space="preserve"> Le code de la sécurité sociale est ainsi modifié :
@@ -430,26 +376,10 @@
   « Art. L. 241-13. – I. – Toute heure supplémentaire effectuée par les salariés mentionnés au I de l’article L. 137-16 ouvre droit à une déduction forfaitaire des charges patronales à hauteur d’un montant fixé par décret. Ce montant peut être majoré dans les entreprises employant au plus vingt salariés »</t>
   </si>
   <si>
-    <t>- 1 code : Le code de la sécurité sociale 
-- 2 experts : Marie Faugeron et Marin Guédo-Guilloteau
-- 1 mot clé exposé des motifs : charges patronales
-- 1 expert : Marie Faugeron</t>
-  </si>
-  <si>
-    <t>- 2 codes : Le code général des impôts, le code du service national 
-- 2 experts : Julien Dauce, Nathan Soto
-- 3 mot-clés : composants de salaire, organisme de protection sociale, composantes salariales
-- 2 experts : Julien Dauce, Nathan Soto</t>
-  </si>
-  <si>
     <t>Rien ici</t>
   </si>
   <si>
     <t>un organisme de protection sociale pour Nathan</t>
-  </si>
-  <si>
-    <t>- 1 mot-clé : organisme de protection sociale
-- 1 expert : Nathan Soto</t>
   </si>
   <si>
     <t>I. – À la fin du I de l’article 1635 bis du code général des impôts, les mots : « et dans une limite annuelle égale à 7 500 € » sont supprimés.
@@ -497,9 +427,6 @@
     <t>Cet amendement d’appel vise à attirer l’attention sur l’Etablissement Français du Sang, grand absent du Ploi de financement de la sécurité sociale.</t>
   </si>
   <si>
-    <t>Charlotte Legresy</t>
-  </si>
-  <si>
     <t>charlotte.legresy@sante.gouv.fr</t>
   </si>
   <si>
@@ -517,24 +444,97 @@
     <t>charges patronales</t>
   </si>
   <si>
-    <t>- 1 mot clé exposé des motifs : charges patronales
-- 1 expert : Marie Faugeron</t>
-  </si>
-  <si>
     <t>II. – La charge pour l’État et les collectivités territoriales est compensée par la création d’une taxe additionnelle à l’accise sur les bidules prévue au chapitre IV du titre Ier du livre III du code des impositions sur les biens et services.</t>
   </si>
   <si>
+    <t>nathan soto</t>
+  </si>
+  <si>
+    <t>- 1 mot-clé : organisme de protection sociale
+- 1 expert : nathan soto</t>
+  </si>
+  <si>
+    <t>marin guédo-guilloteau</t>
+  </si>
+  <si>
+    <t>julien dauce</t>
+  </si>
+  <si>
     <t xml:space="preserve">- 2 codes : Le code général des impôts, le code du service national 
-- 2 experts : Julien Dauce, Nathan Soto
+- 2 experts : julien dauce, nathan soto
+- Pas de mot clé </t>
+  </si>
+  <si>
+    <t xml:space="preserve">- 2 codes : Le code général des impôts, le code du service national 
+- 2 experts : julien dauce, nathan soto
+- 1 mot-clé : composants de salaire
+- 1 expert </t>
+  </si>
+  <si>
+    <t>- 2 codes : Le code général des impôts, le code du service national 
+- 2 experts : julien dauce, nathan soto
+- 2 mot-clés : composants de salaire, organisme de protection sociale
+- 2 experts : julien dauce, nathan soto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- 2 codes : Le code général des impôts, le code du service national 
+- 2 experts : julien dauce, nathan soto
+- 2 mot-clés : composants de salaire, tabac
+- 2 ème mot clé dans une phrase ignorée 
+- 1 expert </t>
+  </si>
+  <si>
+    <t xml:space="preserve">- 2 codes : Le code général des impôts, le code du service national 
+- 2 experts : julien dauce, nathan soto
 - 1 mot-clés : composants de salaire (exposé amdt)
 - 1 expert </t>
+  </si>
+  <si>
+    <t>- 2 codes : Le code général des impôts, le code du service national 
+- 2 experts : julien dauce, nathan soto
+- 3 mot-clés : composants de salaire, organisme de protection sociale, composantes salariales
+- 2 experts : julien dauce, nathan soto</t>
+  </si>
+  <si>
+    <t>marie faugeron</t>
+  </si>
+  <si>
+    <t>- 1 code : Le code de la sécurité sociale 
+- 2 experts : marie faugeron et marin guédo-guilloteau
+- 1 mot clé : cotisations de l'employeur
+- 1 expert : marie faugeron</t>
+  </si>
+  <si>
+    <t>- 1 code : Le code de la sécurité sociale 
+- 2 experts : marie faugeron et marin guédo-guilloteau
+- 1 mot clé exposé des motifs : charges patronales
+- 1 expert : marie faugeron</t>
+  </si>
+  <si>
+    <t>- 1 mot clé exposé des motifs : charges patronales
+- 1 expert : marie faugeron</t>
+  </si>
+  <si>
+    <t>etienne barraud</t>
+  </si>
+  <si>
+    <t>jean-michel montant</t>
+  </si>
+  <si>
+    <t>- Autres montants mais on ne souhaite pas les voir attribués à jean-michel montant puisque ce ne sont pas des montants M ou Z</t>
+  </si>
+  <si>
+    <t>charlotte legresy</t>
+  </si>
+  <si>
+    <t>margot cavely</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -582,6 +582,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -617,7 +624,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -645,6 +652,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -896,7 +904,7 @@
         <v>6</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>124</v>
+        <v>108</v>
       </c>
       <c r="I1" s="2" t="s">
         <v>7</v>
@@ -922,13 +930,13 @@
         <v>11</v>
       </c>
       <c r="G2" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="I2" s="5" t="s">
         <v>12</v>
-      </c>
-      <c r="H2" s="4" t="s">
-        <v>120</v>
-      </c>
-      <c r="I2" s="5" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -939,10 +947,10 @@
         <v>2</v>
       </c>
       <c r="C3" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" s="4" t="s">
         <v>14</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>15</v>
       </c>
       <c r="E3" s="4" t="s">
         <v>10</v>
@@ -951,13 +959,13 @@
         <v>11</v>
       </c>
       <c r="G3" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="I3" s="5" t="s">
         <v>12</v>
-      </c>
-      <c r="H3" s="4" t="s">
-        <v>120</v>
-      </c>
-      <c r="I3" s="5" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -968,10 +976,10 @@
         <v>3</v>
       </c>
       <c r="C4" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" s="4" t="s">
         <v>16</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>17</v>
       </c>
       <c r="E4" s="4" t="s">
         <v>10</v>
@@ -980,13 +988,13 @@
         <v>11</v>
       </c>
       <c r="G4" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="I4" s="5" t="s">
         <v>12</v>
-      </c>
-      <c r="H4" s="4" t="s">
-        <v>120</v>
-      </c>
-      <c r="I4" s="5" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -997,10 +1005,10 @@
         <v>4</v>
       </c>
       <c r="C5" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D5" s="4" t="s">
         <v>18</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>19</v>
       </c>
       <c r="E5" s="4" t="s">
         <v>10</v>
@@ -1009,13 +1017,13 @@
         <v>11</v>
       </c>
       <c r="G5" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="I5" s="5" t="s">
         <v>12</v>
-      </c>
-      <c r="H5" s="4" t="s">
-        <v>120</v>
-      </c>
-      <c r="I5" s="5" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -1026,10 +1034,10 @@
         <v>5</v>
       </c>
       <c r="C6" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D6" s="4" t="s">
         <v>20</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>21</v>
       </c>
       <c r="E6" s="4" t="s">
         <v>10</v>
@@ -1038,13 +1046,13 @@
         <v>11</v>
       </c>
       <c r="G6" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="I6" s="5" t="s">
         <v>12</v>
-      </c>
-      <c r="H6" s="4" t="s">
-        <v>120</v>
-      </c>
-      <c r="I6" s="5" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="7" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -1055,10 +1063,10 @@
         <v>6</v>
       </c>
       <c r="C7" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D7" s="4" t="s">
         <v>22</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>23</v>
       </c>
       <c r="E7" s="4" t="s">
         <v>10</v>
@@ -1067,13 +1075,13 @@
         <v>11</v>
       </c>
       <c r="G7" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="I7" s="5" t="s">
         <v>12</v>
-      </c>
-      <c r="H7" s="4" t="s">
-        <v>120</v>
-      </c>
-      <c r="I7" s="5" t="s">
-        <v>13</v>
       </c>
       <c r="J7" s="3"/>
       <c r="K7" s="3"/>
@@ -1103,25 +1111,25 @@
         <v>7</v>
       </c>
       <c r="C8" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D8" s="4" t="s">
         <v>24</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>25</v>
       </c>
       <c r="E8" s="4" t="s">
         <v>10</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>27</v>
+        <v>128</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>121</v>
+        <v>105</v>
       </c>
       <c r="I8" s="5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="J8" s="3"/>
       <c r="K8" s="3"/>
@@ -1151,25 +1159,25 @@
         <v>8</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="E9" s="4" t="s">
         <v>10</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>27</v>
+        <v>128</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>121</v>
+        <v>105</v>
       </c>
       <c r="I9" s="5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="J9" s="3"/>
       <c r="K9" s="3"/>
@@ -1199,25 +1207,25 @@
         <v>9</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="E10" s="4" t="s">
         <v>10</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>33</v>
+        <v>120</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>121</v>
+        <v>105</v>
       </c>
       <c r="I10" s="5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="J10" s="3"/>
       <c r="K10" s="3"/>
@@ -1247,25 +1255,25 @@
         <v>10</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E11" s="4" t="s">
         <v>10</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>37</v>
+        <v>118</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>122</v>
+        <v>106</v>
       </c>
       <c r="I11" s="5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="J11" s="3"/>
       <c r="K11" s="3"/>
@@ -1295,25 +1303,25 @@
         <v>11</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="E12" s="4" t="s">
         <v>10</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>37</v>
+        <v>118</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>122</v>
+        <v>106</v>
       </c>
       <c r="I12" s="5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="J12" s="3"/>
       <c r="K12" s="3"/>
@@ -1343,25 +1351,25 @@
         <v>12</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="E13" s="4" t="s">
         <v>10</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>37</v>
+        <v>118</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>122</v>
+        <v>106</v>
       </c>
       <c r="I13" s="5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="J13" s="3"/>
       <c r="K13" s="3"/>
@@ -1391,25 +1399,25 @@
         <v>13</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="E14" s="4" t="s">
         <v>10</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>37</v>
+        <v>118</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>122</v>
+        <v>106</v>
       </c>
       <c r="I14" s="5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="J14" s="3"/>
       <c r="K14" s="3"/>
@@ -1439,25 +1447,25 @@
         <v>14</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="E15" s="4" t="s">
         <v>10</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>37</v>
+        <v>118</v>
       </c>
       <c r="H15" s="4" t="s">
-        <v>122</v>
+        <v>106</v>
       </c>
       <c r="I15" s="5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="J15" s="3"/>
       <c r="M15" s="3"/>
@@ -1485,25 +1493,25 @@
         <v>15</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="E16" s="4" t="s">
         <v>10</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>37</v>
+        <v>118</v>
       </c>
       <c r="H16" s="4" t="s">
-        <v>122</v>
+        <v>106</v>
       </c>
       <c r="I16" s="5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="J16" s="3"/>
       <c r="K16" s="3"/>
@@ -1533,25 +1541,25 @@
         <v>16</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="E17" s="4" t="s">
         <v>10</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>37</v>
+        <v>118</v>
       </c>
       <c r="H17" s="4" t="s">
-        <v>122</v>
+        <v>106</v>
       </c>
       <c r="I17" s="5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="J17" s="3"/>
       <c r="K17" s="3"/>
@@ -1581,25 +1589,25 @@
         <v>17</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="E18" s="4" t="s">
         <v>10</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>37</v>
+        <v>118</v>
       </c>
       <c r="H18" s="4" t="s">
-        <v>122</v>
+        <v>106</v>
       </c>
       <c r="I18" s="5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="J18" s="3"/>
       <c r="K18" s="3"/>
@@ -1629,25 +1637,25 @@
         <v>18</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="E19" s="4" t="s">
         <v>10</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>27</v>
+        <v>128</v>
       </c>
       <c r="H19" s="4" t="s">
-        <v>121</v>
+        <v>105</v>
       </c>
       <c r="I19" s="5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="20" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -1658,25 +1666,25 @@
         <v>19</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="E20" s="4" t="s">
         <v>10</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>37</v>
+        <v>118</v>
       </c>
       <c r="H20" s="4" t="s">
-        <v>122</v>
+        <v>106</v>
       </c>
       <c r="I20" s="5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="21" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -1687,25 +1695,25 @@
         <v>20</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="E21" s="4" t="s">
         <v>10</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="G21" s="5" t="s">
-        <v>37</v>
+        <v>118</v>
       </c>
       <c r="H21" s="4" t="s">
-        <v>122</v>
+        <v>106</v>
       </c>
       <c r="I21" s="5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="22" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -1716,25 +1724,25 @@
         <v>21</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="E22" s="4" t="s">
         <v>10</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>37</v>
+        <v>118</v>
       </c>
       <c r="H22" s="4" t="s">
-        <v>122</v>
+        <v>106</v>
       </c>
       <c r="I22" s="5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="23" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -1745,25 +1753,25 @@
         <v>22</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="E23" s="4" t="s">
         <v>10</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="G23" s="5" t="s">
-        <v>63</v>
+        <v>136</v>
       </c>
       <c r="H23" s="4" t="s">
-        <v>121</v>
+        <v>105</v>
       </c>
       <c r="I23" s="5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="24" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -1774,25 +1782,25 @@
         <v>23</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="E24" s="4" t="s">
         <v>10</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="G24" s="5" t="s">
-        <v>37</v>
+        <v>118</v>
       </c>
       <c r="H24" s="4" t="s">
-        <v>122</v>
+        <v>106</v>
       </c>
       <c r="I24" s="5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="25" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -1803,25 +1811,25 @@
         <v>24</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="E25" s="4" t="s">
         <v>10</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G25" s="5" t="s">
-        <v>27</v>
+        <v>128</v>
       </c>
       <c r="H25" s="4" t="s">
-        <v>121</v>
+        <v>105</v>
       </c>
       <c r="I25" s="5" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
     </row>
     <row r="26" spans="1:28" ht="32" x14ac:dyDescent="0.2">
@@ -1832,25 +1840,25 @@
         <v>25</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="E26" s="4" t="s">
         <v>10</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="G26" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="H26" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="I26" s="5" t="s">
         <v>63</v>
-      </c>
-      <c r="H26" s="4" t="s">
-        <v>121</v>
-      </c>
-      <c r="I26" s="5" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="27" spans="1:28" ht="32" x14ac:dyDescent="0.2">
@@ -1861,25 +1869,25 @@
         <v>26</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="E27" s="4" t="s">
         <v>10</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="G27" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="H27" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="I27" s="5" t="s">
         <v>63</v>
-      </c>
-      <c r="H27" s="4" t="s">
-        <v>121</v>
-      </c>
-      <c r="I27" s="5" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="28" spans="1:28" ht="32" x14ac:dyDescent="0.2">
@@ -1890,25 +1898,25 @@
         <v>27</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="E28" s="4" t="s">
         <v>10</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G28" s="5" t="s">
-        <v>27</v>
+        <v>128</v>
       </c>
       <c r="H28" s="4" t="s">
-        <v>121</v>
+        <v>105</v>
       </c>
       <c r="I28" s="5" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
     </row>
     <row r="29" spans="1:28" ht="48" x14ac:dyDescent="0.2">
@@ -1919,25 +1927,25 @@
         <v>28</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="E29" s="4" t="s">
         <v>10</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G29" s="5" t="s">
-        <v>27</v>
+        <v>128</v>
       </c>
       <c r="H29" s="4" t="s">
-        <v>121</v>
+        <v>105</v>
       </c>
       <c r="I29" s="5" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
     </row>
     <row r="30" spans="1:28" ht="64" x14ac:dyDescent="0.2">
@@ -1948,10 +1956,10 @@
         <v>29</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="E30" s="4" t="s">
         <v>10</v>
@@ -1960,13 +1968,13 @@
         <v>11</v>
       </c>
       <c r="G30" s="8" t="s">
-        <v>12</v>
+        <v>121</v>
       </c>
       <c r="H30" s="4" t="s">
-        <v>120</v>
+        <v>104</v>
       </c>
       <c r="I30" s="5" t="s">
-        <v>77</v>
+        <v>122</v>
       </c>
     </row>
     <row r="31" spans="1:28" ht="48" x14ac:dyDescent="0.2">
@@ -1977,25 +1985,25 @@
         <v>30</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="E31" s="4" t="s">
         <v>10</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G31" s="5" t="s">
-        <v>27</v>
+        <v>128</v>
       </c>
       <c r="H31" s="4" t="s">
-        <v>121</v>
+        <v>105</v>
       </c>
       <c r="I31" s="5" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
     </row>
     <row r="32" spans="1:28" ht="144" x14ac:dyDescent="0.2">
@@ -2006,10 +2014,10 @@
         <v>31</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="D32" s="7" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="E32" s="4" t="s">
         <v>10</v>
@@ -2018,13 +2026,13 @@
         <v>11</v>
       </c>
       <c r="G32" s="8" t="s">
-        <v>12</v>
+        <v>121</v>
       </c>
       <c r="H32" s="4" t="s">
-        <v>120</v>
+        <v>104</v>
       </c>
       <c r="I32" s="5" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
     </row>
     <row r="33" spans="1:9" ht="112" x14ac:dyDescent="0.2">
@@ -2035,25 +2043,25 @@
         <v>32</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="E33" s="4" t="s">
         <v>10</v>
       </c>
       <c r="F33" s="4" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="G33" s="5" t="s">
-        <v>90</v>
+        <v>132</v>
       </c>
       <c r="H33" s="4" t="s">
-        <v>123</v>
+        <v>107</v>
       </c>
       <c r="I33" s="5" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
     </row>
     <row r="34" spans="1:9" ht="144" x14ac:dyDescent="0.2">
@@ -2064,25 +2072,25 @@
         <v>33</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="D34" s="7" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="E34" s="4" t="s">
         <v>10</v>
       </c>
       <c r="F34" s="4" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="G34" s="5" t="s">
-        <v>90</v>
+        <v>132</v>
       </c>
       <c r="H34" s="4" t="s">
-        <v>123</v>
+        <v>107</v>
       </c>
       <c r="I34" s="5" t="s">
-        <v>91</v>
+        <v>84</v>
       </c>
     </row>
     <row r="35" spans="1:9" ht="240" x14ac:dyDescent="0.2">
@@ -2093,25 +2101,25 @@
         <v>34</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>92</v>
+        <v>85</v>
       </c>
       <c r="D35" s="7" t="s">
-        <v>93</v>
+        <v>86</v>
       </c>
       <c r="E35" s="4" t="s">
         <v>10</v>
       </c>
       <c r="F35" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G35" s="5" t="s">
-        <v>27</v>
+        <v>128</v>
       </c>
       <c r="H35" s="4" t="s">
-        <v>121</v>
+        <v>105</v>
       </c>
       <c r="I35" s="5" t="s">
-        <v>94</v>
+        <v>129</v>
       </c>
     </row>
     <row r="36" spans="1:9" ht="144" x14ac:dyDescent="0.2">
@@ -2122,10 +2130,10 @@
         <v>35</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="D36" s="7" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="E36" s="4" t="s">
         <v>10</v>
@@ -2134,13 +2142,13 @@
         <v>11</v>
       </c>
       <c r="G36" s="8" t="s">
-        <v>12</v>
+        <v>121</v>
       </c>
       <c r="H36" s="4" t="s">
-        <v>120</v>
+        <v>104</v>
       </c>
       <c r="I36" s="5" t="s">
-        <v>97</v>
+        <v>123</v>
       </c>
     </row>
     <row r="37" spans="1:9" ht="144" x14ac:dyDescent="0.2">
@@ -2151,10 +2159,10 @@
         <v>36</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>98</v>
+        <v>89</v>
       </c>
       <c r="D37" s="7" t="s">
-        <v>99</v>
+        <v>90</v>
       </c>
       <c r="E37" s="4" t="s">
         <v>10</v>
@@ -2163,13 +2171,13 @@
         <v>11</v>
       </c>
       <c r="G37" s="8" t="s">
-        <v>12</v>
+        <v>121</v>
       </c>
       <c r="H37" s="4" t="s">
-        <v>120</v>
+        <v>104</v>
       </c>
       <c r="I37" s="5" t="s">
-        <v>100</v>
+        <v>124</v>
       </c>
     </row>
     <row r="38" spans="1:9" ht="208" x14ac:dyDescent="0.2">
@@ -2180,10 +2188,10 @@
         <v>37</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>101</v>
+        <v>91</v>
       </c>
       <c r="D38" s="7" t="s">
-        <v>102</v>
+        <v>92</v>
       </c>
       <c r="E38" s="4" t="s">
         <v>10</v>
@@ -2192,13 +2200,13 @@
         <v>11</v>
       </c>
       <c r="G38" s="8" t="s">
-        <v>12</v>
+        <v>121</v>
       </c>
       <c r="H38" s="4" t="s">
-        <v>120</v>
+        <v>104</v>
       </c>
       <c r="I38" s="5" t="s">
-        <v>103</v>
+        <v>125</v>
       </c>
     </row>
     <row r="39" spans="1:9" ht="208" x14ac:dyDescent="0.2">
@@ -2209,10 +2217,10 @@
         <v>38</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>101</v>
+        <v>91</v>
       </c>
       <c r="D39" s="7" t="s">
-        <v>104</v>
+        <v>93</v>
       </c>
       <c r="E39" s="4" t="s">
         <v>10</v>
@@ -2221,13 +2229,13 @@
         <v>11</v>
       </c>
       <c r="G39" s="8" t="s">
-        <v>12</v>
+        <v>121</v>
       </c>
       <c r="H39" s="4" t="s">
-        <v>120</v>
+        <v>104</v>
       </c>
       <c r="I39" s="5" t="s">
-        <v>103</v>
+        <v>125</v>
       </c>
     </row>
     <row r="40" spans="1:9" ht="16" x14ac:dyDescent="0.2">
@@ -2238,25 +2246,25 @@
         <v>39</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>101</v>
+        <v>91</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>105</v>
+        <v>94</v>
       </c>
       <c r="E40" s="4" t="s">
         <v>10</v>
       </c>
       <c r="F40" s="9" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="G40" s="5" t="s">
-        <v>107</v>
+        <v>133</v>
       </c>
       <c r="H40" s="4" t="s">
-        <v>120</v>
+        <v>104</v>
       </c>
       <c r="I40" s="5" t="s">
-        <v>108</v>
+        <v>96</v>
       </c>
     </row>
     <row r="41" spans="1:9" ht="48" x14ac:dyDescent="0.2">
@@ -2267,25 +2275,25 @@
         <v>40</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>101</v>
+        <v>91</v>
       </c>
       <c r="D41" s="4" t="s">
-        <v>109</v>
+        <v>97</v>
       </c>
       <c r="E41" s="4" t="s">
         <v>10</v>
       </c>
       <c r="F41" s="9" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="G41" s="5" t="s">
-        <v>90</v>
+        <v>132</v>
       </c>
       <c r="H41" s="4" t="s">
-        <v>123</v>
+        <v>107</v>
       </c>
       <c r="I41" s="5" t="s">
-        <v>110</v>
+        <v>134</v>
       </c>
     </row>
     <row r="42" spans="1:9" ht="112" x14ac:dyDescent="0.2">
@@ -2296,25 +2304,25 @@
         <v>41</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>92</v>
+        <v>85</v>
       </c>
       <c r="D42" s="7" t="s">
-        <v>111</v>
+        <v>98</v>
       </c>
       <c r="E42" s="4" t="s">
-        <v>112</v>
+        <v>99</v>
       </c>
       <c r="F42" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G42" s="5" t="s">
-        <v>27</v>
+        <v>128</v>
       </c>
       <c r="H42" s="4" t="s">
-        <v>121</v>
+        <v>105</v>
       </c>
       <c r="I42" s="5" t="s">
-        <v>113</v>
+        <v>130</v>
       </c>
     </row>
     <row r="43" spans="1:9" ht="176" x14ac:dyDescent="0.2">
@@ -2325,25 +2333,25 @@
         <v>42</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>101</v>
+        <v>91</v>
       </c>
       <c r="D43" s="7" t="s">
-        <v>119</v>
+        <v>103</v>
       </c>
       <c r="E43" s="4" t="s">
-        <v>135</v>
+        <v>117</v>
       </c>
       <c r="F43" s="7" t="s">
         <v>11</v>
       </c>
       <c r="G43" s="8" t="s">
-        <v>12</v>
+        <v>121</v>
       </c>
       <c r="H43" s="4" t="s">
-        <v>120</v>
+        <v>104</v>
       </c>
       <c r="I43" s="5" t="s">
-        <v>136</v>
+        <v>126</v>
       </c>
     </row>
     <row r="44" spans="1:9" ht="144" x14ac:dyDescent="0.2">
@@ -2354,25 +2362,25 @@
         <v>43</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>98</v>
+        <v>89</v>
       </c>
       <c r="D44" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="E44" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="F44" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="G44" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="E44" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="F44" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="G44" s="5" t="s">
-        <v>37</v>
-      </c>
       <c r="H44" s="4" t="s">
-        <v>122</v>
+        <v>106</v>
       </c>
       <c r="I44" s="5" t="s">
-        <v>114</v>
+        <v>127</v>
       </c>
     </row>
     <row r="45" spans="1:9" ht="32" x14ac:dyDescent="0.2">
@@ -2383,25 +2391,25 @@
         <v>44</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>98</v>
+        <v>89</v>
       </c>
       <c r="D45" s="7" t="s">
-        <v>115</v>
+        <v>100</v>
       </c>
       <c r="E45" s="4" t="s">
-        <v>116</v>
+        <v>101</v>
       </c>
       <c r="F45" s="4" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="G45" s="5" t="s">
-        <v>37</v>
+        <v>118</v>
       </c>
       <c r="H45" s="4" t="s">
-        <v>122</v>
+        <v>106</v>
       </c>
       <c r="I45" s="5" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
     </row>
     <row r="46" spans="1:9" ht="64" x14ac:dyDescent="0.2">
@@ -2412,25 +2420,25 @@
         <v>45</v>
       </c>
       <c r="C46" t="s">
-        <v>125</v>
+        <v>109</v>
       </c>
       <c r="D46" t="s">
-        <v>126</v>
+        <v>110</v>
       </c>
       <c r="E46" t="s">
-        <v>127</v>
+        <v>111</v>
       </c>
       <c r="F46" s="10" t="s">
-        <v>129</v>
-      </c>
-      <c r="G46" t="s">
-        <v>128</v>
+        <v>112</v>
+      </c>
+      <c r="G46" s="11" t="s">
+        <v>135</v>
       </c>
       <c r="H46" s="4" t="s">
-        <v>130</v>
+        <v>113</v>
       </c>
       <c r="I46" s="5" t="s">
-        <v>131</v>
+        <v>114</v>
       </c>
     </row>
     <row r="47" spans="1:9" ht="32" x14ac:dyDescent="0.2">
@@ -2441,25 +2449,25 @@
         <v>46</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>92</v>
+        <v>85</v>
       </c>
       <c r="D47" s="7" t="s">
-        <v>132</v>
+        <v>115</v>
       </c>
       <c r="E47" s="4" t="s">
-        <v>133</v>
+        <v>116</v>
       </c>
       <c r="F47" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G47" s="5" t="s">
-        <v>27</v>
+        <v>128</v>
       </c>
       <c r="H47" s="4" t="s">
-        <v>121</v>
+        <v>105</v>
       </c>
       <c r="I47" s="5" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.2">

</xml_diff>